<commit_message>
Enhance ExcelConfigBootstrap and ExcelConfigReader to improve request body handling; implement additional methods for better JSON data processing and response management, ensuring more efficient data retrieval.
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -80,10 +80,10 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-18T13:59:06.9035897Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-18T13:59:10.4046459Z</x:t>
+    <x:t>2026-06-18T14:05:11.1761811Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-18T14:05:13.8988075Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
Excel implemetation done partially
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -80,10 +80,10 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-18T14:05:11.1761811Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-18T14:05:13.8988075Z</x:t>
+    <x:t>2026-06-18T14:17:31.3899859Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-18T14:17:37.2751996Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
deleted the json file
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -80,10 +80,10 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-18T14:17:31.3899859Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-18T14:17:37.2751996Z</x:t>
+    <x:t>2026-06-18T14:35:58.2488621Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-18T14:36:04.2925489Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
Added Feature file Address
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -80,10 +80,10 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-18T14:35:58.2488621Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-18T14:36:04.2925489Z</x:t>
+    <x:t>2026-06-19T13:23:32.8023305Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-19T13:23:39.4441167Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
updated Expired token value and key changes done
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-06T20:22:03.3397368Z</x:t>
+    <x:t>2026-07-13T13:15:16.3071586Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-06T10:18:01.1205500Z</x:t>
+    <x:t>2026-07-13T13:14:31.8760999Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-09T20:08:08.0089810Z</x:t>
+    <x:t>2026-07-13T14:31:44.9707385Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
Address.feature , Businesunit.feature added
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-13T13:15:16.3071586Z</x:t>
+    <x:t>2026-08-03T13:57:34.0116371Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-13T13:14:31.8760999Z</x:t>
+    <x:t>2026-07-15T13:39:10.2151736Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-14T11:40:34.5361599Z</x:t>
+    <x:t>2026-08-03T13:57:48.3713566Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
Update Framework name and Feature Title and added new feature
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-08-03T13:57:34.0116371Z</x:t>
+    <x:t>2026-08-08T10:26:03.2318906Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-15T13:39:10.2151736Z</x:t>
+    <x:t>2026-08-08T10:25:52.2925007Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-08-03T13:57:48.3713566Z</x:t>
+    <x:t>2026-08-08T10:26:04.8705957Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>